<commit_message>
New inferences on Jesuit Entry
</commit_message>
<xml_diff>
--- a/inferences/jesuita-entrada-Coimbra.xlsx
+++ b/inferences/jesuita-entrada-Coimbra.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,11 +499,6 @@
           <t>morte</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>jesuita-entrada.extra_info</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -556,11 +551,6 @@
           <t>?</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}, 'obs': {'kleio_element_name': 'obs', 'kleio_element_class': 'obs', 'entity_attr_name': 'obs', 'entity_column_class': 'obs'}}</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -623,11 +613,6 @@
           <t>Goa</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>{'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}}</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -690,11 +675,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -757,11 +737,6 @@
           <t>Negapatam</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'já é padre'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -824,11 +799,6 @@
           <t>Goa</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>{'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}}</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -891,11 +861,6 @@
           <t>[A caminho do Japão]</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -956,11 +921,6 @@
       <c r="N8" t="inlineStr">
         <is>
           <t>Macau</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -1013,11 +973,6 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1080,11 +1035,6 @@
           <t>[No mar, a caminho de Malaca]</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1147,11 +1097,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Domingues &amp; O Neil, IV: 2645. MMHM:p.226', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 15600325 ou Coimbra, 25-03-1560 MMHM'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1214,11 +1159,6 @@
           <t>Goa (Colégio Novo)</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1279,11 +1219,6 @@
       <c r="N13" t="inlineStr">
         <is>
           <t>Macau (colégio)</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Está no "Catálogo delos Padres y Hermanos dela Provincia de Portugal a 12 de Enero de 1579",Lus. 39 p.3v, nos estudantes de Filosofia do segundo curso', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -1336,11 +1271,6 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Schutte, Monumenta historica japoniae I.,p.1180', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1403,11 +1333,6 @@
           <t>Shiuchow</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 "Catálogo delos Padres y Hermanos dela Provincia de Portugal a 12 de Enero de 1579" Lus. 39, 3v, estudante de filosofia, 1ºcurso', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1470,11 +1395,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1537,11 +1457,6 @@
           <t>Hang-tcheou</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Em Coimbra no ano de 1582 segundo a Carta Annua de 1623 BA', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}, 'obs': {'kleio_element_name': 'obs', 'kleio_element_class': 'obs', 'entity_attr_name': 'obs', 'entity_column_class': 'obs'}}</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1604,11 +1519,6 @@
           <t>Japão</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 MMHM:p.94 (ARSI Japsin 35 13)', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1671,11 +1581,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1738,11 +1643,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1805,11 +1705,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Segundo Dominguez &amp; O Neil, V.III,p.2961. Franco Imagem...Coimbra,II,4,c.36,p.575', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -1872,11 +1767,6 @@
           <t>Nagasaki</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -1939,11 +1829,6 @@
           <t>Cantão</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2006,11 +1891,6 @@
           <t>Japão</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -2073,11 +1953,6 @@
           <t>Edo</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412([Schütte, 1975, p. 1321] Sebastião Vieira, nasc Castro de Aire, Lamego, E. Coimbra 3-2-1591', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -2140,11 +2015,6 @@
           <t>Hangchow</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Segungo Dominguez, J. M., &amp; O’Neill, C. (2001) II, 1113', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -2207,11 +2077,6 @@
           <t>Nanquim</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -2274,11 +2139,6 @@
           <t>Goa</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': 'Franco, 1717, p. 375, Sweet, 20216, p.27 @wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -2341,11 +2201,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Dehergne não especifica local, Brockey estudos Filosofia e Teologia em Coimbra', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -2408,11 +2263,6 @@
           <t>Foochow, Fukien</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 (Franco, 1719, t.II, p. 612)', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 16090502 reentrou em 1611 não se sabe onde'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -2475,11 +2325,6 @@
           <t>[Perto de Hainan]</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '[Adicionado a partir de Franco, Imagem...Coimbra, II, 522] @wikidata:Q45412', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'MMHM:p.8'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -2542,11 +2387,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 """Franco, Imagem...Coimbra, v.2 p.616; Barbosa Machado, v.3"""', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -2609,11 +2449,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': "@wikidata:Q45412 MMHM:p.205 (Sebastian da Maia, da Maya, d'Amaya)", 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -2676,11 +2511,6 @@
           <t>Pequim</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Segundo Louis Buglio 1688', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -2743,11 +2573,6 @@
           <t>Costa da Cochinchina</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': "@wikidata:Q45412 MMHM:p.203 (Matias d'Amaia), Schutte, Monumenta historica japoniae I.1234", 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -2808,11 +2633,6 @@
       <c r="N36" t="inlineStr">
         <is>
           <t>Macau</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Segundo Schütte, p.1174', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -2865,11 +2685,6 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Ver Brockey, p.230 cit. Carta de A.P. a Viteleschi, de Coimbra, 26 Agosto 1640', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -2932,11 +2747,6 @@
           <t>Nanquim</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -2999,11 +2809,6 @@
           <t>Foochow (Fou-tcheou fou, Fukien)</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412 Brockey, cap.6 n.95', 'original': '?'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}, 'obs': {'kleio_element_name': 'obs', 'kleio_element_class': 'obs', 'entity_attr_name': 'obs', 'entity_column_class': 'obs'}}</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -3066,11 +2871,6 @@
           <t>[No mar, depois do Cabo da Boa Esperança]</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
@@ -3133,11 +2933,6 @@
           <t>Pequim</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -3198,11 +2993,6 @@
       <c r="N42" t="inlineStr">
         <is>
           <t>Goa</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 16630325'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -3247,11 +3037,6 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -3314,11 +3099,6 @@
           <t>Nanquim</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 16690519'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -3381,11 +3161,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
@@ -3448,11 +3223,6 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
@@ -3515,11 +3285,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
@@ -3582,11 +3347,6 @@
           <t>Coimbra</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -3649,11 +3409,6 @@
           <t>Macau</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
@@ -3716,11 +3471,6 @@
           <t>Tonquim</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
@@ -3781,11 +3531,6 @@
       <c r="N51" t="inlineStr">
         <is>
           <t>Macau</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -3838,11 +3583,6 @@
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -3893,11 +3633,6 @@
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
@@ -3960,11 +3695,6 @@
           <t>Pequim</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
@@ -4027,11 +3757,6 @@
           <t>Goa</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 16931016 ou 16931021 ou 16930326'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
@@ -4092,11 +3817,6 @@
       <c r="N56" t="inlineStr">
         <is>
           <t>?</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -4149,11 +3869,6 @@
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
@@ -4214,11 +3929,6 @@
       <c r="N58" t="inlineStr">
         <is>
           <t>?</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>
@@ -4271,11 +3981,6 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date', 'comment': 'ou 17051224'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -4338,11 +4043,6 @@
           <t>Castel Gandolfo</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
@@ -4405,11 +4105,6 @@
           <t>Pequim</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
@@ -4470,11 +4165,6 @@
       <c r="N62" t="inlineStr">
         <is>
           <t>?</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>{'id': {'kleio_element_name': 'id', 'kleio_element_class': 'id', 'entity_attr_name': 'id', 'entity_column_class': 'id'}, 'the_value': {'kleio_element_name': 'valor', 'kleio_element_class': 'value', 'entity_attr_name': 'value', 'entity_column_class': 'value', 'comment': '@wikidata:Q45412'}, 'the_type': {'kleio_element_name': 'tipo', 'kleio_element_class': 'type', 'entity_attr_name': 'type', 'entity_column_class': 'type'}, 'the_date': {'kleio_element_name': 'date', 'kleio_element_class': 'date', 'entity_attr_name': 'date', 'entity_column_class': 'date'}, 'entity': {'kleio_element_name': 'entity', 'kleio_element_class': 'entity', 'entity_attr_name': 'entity', 'entity_column_class': 'entity'}, 'class': {'kleio_element_name': 'class', 'kleio_element_class': 'class', 'entity_attr_name': 'class', 'entity_column_class': 'class'}}</t>
         </is>
       </c>
     </row>

</xml_diff>